<commit_message>
Update Report.py with fixed pages and year routing
</commit_message>
<xml_diff>
--- a/2026-27/CWSN_Student_List_AY_2026-27.xlsx
+++ b/2026-27/CWSN_Student_List_AY_2026-27.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Report_py\2026-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18DA07C8-A340-4648-BCD8-EF8F9253C898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D46AB4-0A4D-46D6-A56A-5A183BDD7AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CWSN Student List" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CWSN Student List'!$A$2:$P$364</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -4015,7 +4018,8 @@
     <col min="6" max="8" width="21" customWidth="1"/>
     <col min="9" max="9" width="41" customWidth="1"/>
     <col min="10" max="13" width="14" customWidth="1"/>
-    <col min="14" max="16" width="20" customWidth="1"/>
+    <col min="14" max="14" width="38.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -9784,7 +9788,7 @@
         <v>501</v>
       </c>
       <c r="N129" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O129" s="2" t="s">
         <v>502</v>
@@ -9834,7 +9838,7 @@
         <v>504</v>
       </c>
       <c r="N130" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O130" s="2" t="s">
         <v>502</v>
@@ -10016,7 +10020,7 @@
         <v>518</v>
       </c>
       <c r="N134" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O134" s="2" t="s">
         <v>502</v>
@@ -10066,7 +10070,7 @@
         <v>520</v>
       </c>
       <c r="N135" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O135" s="2" t="s">
         <v>502</v>
@@ -10116,7 +10120,7 @@
         <v>524</v>
       </c>
       <c r="N136" s="2" t="s">
-        <v>525</v>
+        <v>172</v>
       </c>
     </row>
     <row r="137" spans="1:16" x14ac:dyDescent="0.25">
@@ -10659,7 +10663,7 @@
         <v>559</v>
       </c>
       <c r="N148" s="2" t="s">
-        <v>525</v>
+        <v>172</v>
       </c>
     </row>
     <row r="149" spans="1:15" x14ac:dyDescent="0.25">
@@ -11868,7 +11872,7 @@
         <v>641</v>
       </c>
       <c r="N175" s="2" t="s">
-        <v>525</v>
+        <v>172</v>
       </c>
     </row>
     <row r="176" spans="1:16" x14ac:dyDescent="0.25">
@@ -12268,7 +12272,7 @@
       </c>
       <c r="M184" s="2"/>
       <c r="N184" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O184" s="2" t="s">
         <v>502</v>
@@ -15214,7 +15218,7 @@
         <v>875</v>
       </c>
       <c r="N250" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O250" s="2" t="s">
         <v>502</v>
@@ -15262,7 +15266,7 @@
       </c>
       <c r="M251" s="2"/>
       <c r="N251" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O251" s="2" t="s">
         <v>502</v>
@@ -15312,7 +15316,7 @@
         <v>878</v>
       </c>
       <c r="N252" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O252" s="2" t="s">
         <v>502</v>
@@ -15362,7 +15366,7 @@
         <v>880</v>
       </c>
       <c r="N253" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O253" s="2" t="s">
         <v>502</v>
@@ -15410,7 +15414,7 @@
       </c>
       <c r="M254" s="2"/>
       <c r="N254" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O254" s="2" t="s">
         <v>502</v>
@@ -15460,7 +15464,7 @@
         <v>883</v>
       </c>
       <c r="N255" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O255" s="2" t="s">
         <v>502</v>
@@ -16050,7 +16054,7 @@
         <v>927</v>
       </c>
       <c r="N268" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O268" s="2" t="s">
         <v>502</v>
@@ -16810,7 +16814,7 @@
         <v>976</v>
       </c>
       <c r="N285" s="2" t="s">
-        <v>525</v>
+        <v>172</v>
       </c>
     </row>
     <row r="286" spans="1:15" x14ac:dyDescent="0.25">
@@ -17295,7 +17299,7 @@
       </c>
       <c r="M296" s="2"/>
       <c r="N296" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O296" s="2" t="s">
         <v>502</v>
@@ -17873,7 +17877,7 @@
         <v>1048</v>
       </c>
       <c r="N309" s="2" t="s">
-        <v>525</v>
+        <v>172</v>
       </c>
     </row>
     <row r="310" spans="1:14" x14ac:dyDescent="0.25">
@@ -19453,7 +19457,7 @@
       </c>
       <c r="M345" s="2"/>
       <c r="N345" s="2" t="s">
-        <v>502</v>
+        <v>172</v>
       </c>
       <c r="O345" s="2" t="s">
         <v>502</v>

</xml_diff>